<commit_message>
Stage 8c: AI kick-off proposal in sign-off workbook; provisional drilled length; F-1 check
</commit_message>
<xml_diff>
--- a/outputs/kickoff_signoff.xlsx
+++ b/outputs/kickoff_signoff.xlsx
@@ -30,7 +30,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +40,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F0FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -60,13 +65,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -434,25 +442,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="80" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,15 +535,35 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>proposed_by</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>proposed_approved</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>proposed_depth</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>proposed_reason</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>author_approved</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>author_depth</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>author_note</t>
         </is>
@@ -593,9 +625,27 @@
           <t>window top; a first window (2202-2207 m, 1997-07-26) was abandoned</t>
         </is>
       </c>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>2183</v>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>The 1997-07-29 report states the window milled 2178-2183 m with 19 m of formation drilled below it, so under the rule's first tier the hole leaves the parent at the window bottom, 2183 m; 2178 m (window start) is the second-tier fallback for when no departure depth is stated. The first window (2202-2207 m, 1997-07-26) was abandoned and is not the kick-off; NOD and the structured field say 2178 m.</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="n"/>
+      <c r="T2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -647,9 +697,27 @@
       </c>
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>2231</v>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>The report states the kick-off depth directly: 'DRESS CMT AND PERFORMED KICK OFF FROM 2231M TO 2277M'. NOD's 2,200 m is not an input to the rule; the only '2200' in the 19 A and 19 B reports is a clock time ('AT 2200 HRS').</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="n"/>
+      <c r="T3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -705,9 +773,27 @@
           <t>NOD has no separate record (its 15/9-19 B record is the B leg)</t>
         </is>
       </c>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>2911</v>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>The parent's last report states departure with a depth: 'COMMENCED DRILLING 8 1/2" HOLE FROM 2911 M AT 15/9-19BT2' (after cement drilled to 2911 m), and the first BT2 report starts at the same depth. Tier 1.</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="n"/>
+      <c r="T4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -763,9 +849,27 @@
           <t>both reports of 1992-12-19 read 'None'</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>1536</v>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Both 1992-12-19 narratives (parent last, sidetrack first) read 'None', so the third tier applies: measured depth at the transition, 1,536 m on both reports. Depth only, no text support; the parent had drilled cement to 1,486 m the day before, so the true departure could be shallower.</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -821,9 +925,27 @@
           <t>event named in the parent's last report; md 2620</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>2620</v>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>The parent's last report says 'Commenced kick off to F-1A' without a depth and its md is 2620 m, so tier 2, event in text with depth from md. NOD agrees at 2,620 m.</t>
+        </is>
+      </c>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -879,9 +1001,27 @@
           <t>event named in the parent's last report; md 2617</t>
         </is>
       </c>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>2617</v>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>The parent's last report says 'Drilled out cement and kicked off well to F-1 B' and its md is 2617 m (2,545 m the day before), so tier 2, event in text with depth from md; the md is the day's deepest point, so the kick-off may be a little shallower (NOD 2,604 m).</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="n"/>
+      <c r="S7" s="4" t="n"/>
+      <c r="T7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -941,9 +1081,27 @@
           <t>new formation (50%) first reported at 1364 m</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>1364</v>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Tier 1: the F-1 B report of 2014-02-22 states '50% formation obtained at 1364 m', the first report of new formation, and F-1 C's first report drills from 1,364 m. 1,355 m is only where time drilling started, the fallback used when no formation depth is stated. NOD agrees at 1,364 m.</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="n"/>
+      <c r="T8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1003,9 +1161,27 @@
           <t>window top</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>428.2</v>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>The window was milled from 421.5 m (top) to 428.2 m (bottom) and the 2009-07-02 report continues to drill formation below it (to 436.5 m), so the stated departure and first new formation are at the window bottom, 428.2 m (NOD 428 m); 421.5 m is the window-start fallback.</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" s="4" t="n"/>
+      <c r="T9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1061,9 +1237,27 @@
           <t>start of oriented drilling out of the cement (TOC 244 m); NOD has no separate record</t>
         </is>
       </c>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>246</v>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>No formation or departure depth is stated, so tier 2: the 2013-03-23 report says oriented drilling out of the cement started at 246 m (top of cement 244 m). 257 m is where the sidetrack was handed over the next day. NOD has no separate record.</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="n"/>
+      <c r="S10" s="4" t="n"/>
+      <c r="T10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1115,9 +1309,27 @@
       </c>
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="3" t="n"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>2586</v>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Tier 1: 'Drilled cement and kicked off to F-11 A at 2586m MD' states the departure depth. NOD 2,578 m.</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="n"/>
+      <c r="S11" s="4" t="n"/>
+      <c r="T11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1177,9 +1389,27 @@
           <t>new formation reported by 2589 m; evidence is an interval 2531 to 2589 m</t>
         </is>
       </c>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>2531</v>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>The only evidence is 'Drilled cement and new formation from 2531 m MD to 2589 m MD': the depth at which new formation is first reported is not separable inside the interval, so the first tier gives no point value; the second tier gives where the kick-off drilling started, 2,531 m. The sidetrack's first report starts at 2,627 m, so 2,589 m is not supported either. NOD 2,586 m and 2,589 m both lie inside the interval, so the uncertainty is about 58 m.</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="n"/>
+      <c r="T12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1235,9 +1465,27 @@
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="n">
+        <v>1381</v>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>'Drilled cement/new formation from 1368 m to 1381 m MD. Initiated kick off of F-15.' puts the start of the kick-off at the end of the interval, 1,381 m, where the sidetrack's first report also starts. NOD agrees at 1,381 m.</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="n"/>
+      <c r="T13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1293,9 +1541,27 @@
         </is>
       </c>
       <c r="M14" s="2" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>3185</v>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Tier 1: 'kicked off at 3185m' states the departure depth; the '50/50 cement/formation' remark relates to 3,210 m, drilled afterwards. NOD agrees at 3,185 m.</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="n"/>
+      <c r="T14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1355,9 +1621,27 @@
           <t>kick-off initiated after cement drilled to 2566 m</t>
         </is>
       </c>
-      <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="3" t="n"/>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>2566</v>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Tier 2: cement was drilled from 2,490 to 2,566 m, then 'Initiated kick off', and no formation or departure depth is stated; 2,575 m (the NOD value) is only where the section had reached by the end of the day.</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="4" t="n"/>
+      <c r="T15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1413,13 +1697,31 @@
           <t>parent set kick-off plug 2013-11-10; child's first report says 'kicked off' without a depth</t>
         </is>
       </c>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>1380</v>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>The sidetrack's first report says 'Drilled cement and kicked off' without a depth, so tier 2 with depth from md: the parent's last report (kick-off plug set the day before) has md 1,380 m. NOD agrees at 1,380 m.</t>
+        </is>
+      </c>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="n"/>
+      <c r="T16" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N2:N16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O16 R2:R16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1433,7 +1735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -1442,7 +1744,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Kick-off sign-off, one row per sidetrack (15). Fill author_approved (Y/N), author_depth (if different) and author_note; the manuscript will use only author-approved depths.</t>
+          <t>Kick-off sign-off, 15 sidetracks. Blue columns = AI PROPOSAL (proposed_by = AI); yellow columns = author (TJ), empty until TJ fills them. The manuscript will use only author-approved depths.</t>
         </is>
       </c>
     </row>
@@ -1456,28 +1758,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rule_tier: T1 = depth stated with new-formation or departure language; T2 = kick-off or window start (window top for windows); T3 = narrative empty (depth sequence).</t>
+          <t>proposed_approved = Y where the proposal equals the current ddr_kickoff_depth_m; N where the evidence or rule does not support the current value, with proposed_depth.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>method: 'depth in text' | 'event in text, depth from md' | 'depth sequence (narrative empty)'.</t>
+          <t>Everything derived from the proposed depths (drilled_length_m, m_per_report_day) is PROVISIONAL until the author columns are filled.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>alternative_depths: other readings of the rule that the evidence allows; they are not applied.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Evidence quotes are 15 words or fewer (cut from the raw narrative, so they can start mid-sentence). NOD = wlbKickOffPoint, snapshot 2026-10-24. Depths in m MD.</t>
+          <t>Quotes are 15 words or fewer. NOD = wlbKickOffPoint, snapshot 2026-10-24. Depths in m MD.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rulings: window-top rule, one spud-offset definition, citations and licence logged; proposals, duration and Fig 4 regenerated
</commit_message>
<xml_diff>
--- a/outputs/kickoff_signoff.xlsx
+++ b/outputs/kickoff_signoff.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:X16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -462,9 +462,13 @@
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="80" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="80" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -555,15 +559,35 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>proposed_by</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>proposed_approved</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>proposed_depth</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>proposed_reason</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>author_approved</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>author_depth</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>author_note</t>
         </is>
@@ -632,20 +656,38 @@
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P2" s="3" t="n">
-        <v>2183</v>
+        <v>2178</v>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>The 1997-07-29 report states the window milled 2178-2183 m with 19 m of formation drilled below it, so under the rule's first tier the hole leaves the parent at the window bottom, 2183 m; 2178 m (window start) is the second-tier fallback for when no departure depth is stated. The first window (2202-2207 m, 1997-07-26) was abandoned and is not the kick-off; NOD and the structured field say 2178 m.</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
+          <t>Casing exit by a milled window: under the rule as ruled by TJ (decision 40) the kick-off is the top of the window, 2,178 m (window milled 2178-2183 m on 1997-07-29; an earlier window at 2,202-2,207 m was abandoned). NOD and the structured mdKickoff also say 2,178 m.</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>2178</v>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>Casing exit by a milled window: under the rule as ruled by TJ (decision 40) the kick-off is the top of the window, 2,178 m (window milled 2178-2183 m on 1997-07-29; an earlier window at 2,202-2,207 m was abandoned). NOD and the structured mdKickoff also say 2,178 m.</t>
+        </is>
+      </c>
+      <c r="V2" s="4" t="n"/>
+      <c r="W2" s="4" t="n"/>
+      <c r="X2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -715,9 +757,27 @@
           <t>The report states the kick-off depth directly: 'DRESS CMT AND PERFORMED KICK OFF FROM 2231M TO 2277M'. NOD's 2,200 m is not an input to the rule; the only '2200' in the 19 A and 19 B reports is a clock time ('AT 2200 HRS').</t>
         </is>
       </c>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>2231</v>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>The report states the kick-off depth directly: 'DRESS CMT AND PERFORMED KICK OFF FROM 2231M TO 2277M'. NOD's 2,200 m is not an input to the rule; the only '2200' in the 19 A and 19 B reports is a clock time ('AT 2200 HRS').</t>
+        </is>
+      </c>
+      <c r="V3" s="4" t="n"/>
+      <c r="W3" s="4" t="n"/>
+      <c r="X3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -791,9 +851,27 @@
           <t>The parent's last report states departure with a depth: 'COMMENCED DRILLING 8 1/2" HOLE FROM 2911 M AT 15/9-19BT2' (after cement drilled to 2911 m), and the first BT2 report starts at the same depth. Tier 1.</t>
         </is>
       </c>
-      <c r="R4" s="4" t="n"/>
-      <c r="S4" s="4" t="n"/>
-      <c r="T4" s="4" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>2911</v>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>The parent's last report states departure with a depth: 'COMMENCED DRILLING 8 1/2" HOLE FROM 2911 M AT 15/9-19BT2' (after cement drilled to 2911 m), and the first BT2 report starts at the same depth. Tier 1.</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="n"/>
+      <c r="W4" s="4" t="n"/>
+      <c r="X4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -867,9 +945,27 @@
           <t>Both 1992-12-19 narratives (parent last, sidetrack first) read 'None', so the third tier applies: measured depth at the transition, 1,536 m on both reports. Depth only, no text support; the parent had drilled cement to 1,486 m the day before, so the true departure could be shallower.</t>
         </is>
       </c>
-      <c r="R5" s="4" t="n"/>
-      <c r="S5" s="4" t="n"/>
-      <c r="T5" s="4" t="n"/>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>1536</v>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>Both 1992-12-19 narratives (parent last, sidetrack first) read 'None', so the third tier applies: measured depth at the transition, 1,536 m on both reports. Depth only, no text support; the parent had drilled cement to 1,486 m the day before, so the true departure could be shallower.</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="n"/>
+      <c r="W5" s="4" t="n"/>
+      <c r="X5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -943,9 +1039,27 @@
           <t>The parent's last report says 'Commenced kick off to F-1A' without a depth and its md is 2620 m, so tier 2, event in text with depth from md. NOD agrees at 2,620 m.</t>
         </is>
       </c>
-      <c r="R6" s="4" t="n"/>
-      <c r="S6" s="4" t="n"/>
-      <c r="T6" s="4" t="n"/>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>2620</v>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>The parent's last report says 'Commenced kick off to F-1A' without a depth and its md is 2620 m, so tier 2, event in text with depth from md. NOD agrees at 2,620 m.</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="n"/>
+      <c r="W6" s="4" t="n"/>
+      <c r="X6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1019,9 +1133,27 @@
           <t>The parent's last report says 'Drilled out cement and kicked off well to F-1 B' and its md is 2617 m (2,545 m the day before), so tier 2, event in text with depth from md; the md is the day's deepest point, so the kick-off may be a little shallower (NOD 2,604 m).</t>
         </is>
       </c>
-      <c r="R7" s="4" t="n"/>
-      <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="n">
+        <v>2617</v>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>The parent's last report says 'Drilled out cement and kicked off well to F-1 B' and its md is 2617 m (2,545 m the day before), so tier 2, event in text with depth from md; the md is the day's deepest point, so the kick-off may be a little shallower (NOD 2,604 m).</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="n"/>
+      <c r="W7" s="4" t="n"/>
+      <c r="X7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1099,9 +1231,27 @@
           <t>Tier 1: the F-1 B report of 2014-02-22 states '50% formation obtained at 1364 m', the first report of new formation, and F-1 C's first report drills from 1,364 m. 1,355 m is only where time drilling started, the fallback used when no formation depth is stated. NOD agrees at 1,364 m.</t>
         </is>
       </c>
-      <c r="R8" s="4" t="n"/>
-      <c r="S8" s="4" t="n"/>
-      <c r="T8" s="4" t="n"/>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="n">
+        <v>1364</v>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>Tier 1: the F-1 B report of 2014-02-22 states '50% formation obtained at 1364 m', the first report of new formation, and F-1 C's first report drills from 1,364 m. 1,355 m is only where time drilling started, the fallback used when no formation depth is stated. NOD agrees at 1,364 m.</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="n"/>
+      <c r="W8" s="4" t="n"/>
+      <c r="X8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1168,20 +1318,38 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P9" s="3" t="n">
-        <v>428.2</v>
+        <v>421.5</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>The window was milled from 421.5 m (top) to 428.2 m (bottom) and the 2009-07-02 report continues to drill formation below it (to 436.5 m), so the stated departure and first new formation are at the window bottom, 428.2 m (NOD 428 m); 421.5 m is the window-start fallback.</t>
-        </is>
-      </c>
-      <c r="R9" s="4" t="n"/>
-      <c r="S9" s="4" t="n"/>
-      <c r="T9" s="4" t="n"/>
+          <t>Casing exit by a milled window: kick-off = top of window, 421.5 m ('Milled 12-1/4" sidetrack window from 421,5 m (top) to 424 m'); the window bottom, 428.2 m, is not used (TJ ruling, decision 40). NOD gives 428 m.</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="n">
+        <v>421.5</v>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>Casing exit by a milled window: kick-off = top of window, 421.5 m ('Milled 12-1/4" sidetrack window from 421,5 m (top) to 424 m'); the window bottom, 428.2 m, is not used (TJ ruling, decision 40). NOD gives 428 m.</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="n"/>
+      <c r="W9" s="4" t="n"/>
+      <c r="X9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1255,9 +1423,27 @@
           <t>No formation or departure depth is stated, so tier 2: the 2013-03-23 report says oriented drilling out of the cement started at 246 m (top of cement 244 m). 257 m is where the sidetrack was handed over the next day. NOD has no separate record.</t>
         </is>
       </c>
-      <c r="R10" s="4" t="n"/>
-      <c r="S10" s="4" t="n"/>
-      <c r="T10" s="4" t="n"/>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="n">
+        <v>246</v>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>No formation or departure depth is stated, so tier 2: the 2013-03-23 report says oriented drilling out of the cement started at 246 m (top of cement 244 m). 257 m is where the sidetrack was handed over the next day. NOD has no separate record.</t>
+        </is>
+      </c>
+      <c r="V10" s="4" t="n"/>
+      <c r="W10" s="4" t="n"/>
+      <c r="X10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1327,9 +1513,27 @@
           <t>Tier 1: 'Drilled cement and kicked off to F-11 A at 2586m MD' states the departure depth. NOD 2,578 m.</t>
         </is>
       </c>
-      <c r="R11" s="4" t="n"/>
-      <c r="S11" s="4" t="n"/>
-      <c r="T11" s="4" t="n"/>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="n">
+        <v>2586</v>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>Tier 1: 'Drilled cement and kicked off to F-11 A at 2586m MD' states the departure depth. NOD 2,578 m.</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="n"/>
+      <c r="W11" s="4" t="n"/>
+      <c r="X11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1396,20 +1600,38 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P12" s="3" t="n">
-        <v>2531</v>
+        <v>2589</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>The only evidence is 'Drilled cement and new formation from 2531 m MD to 2589 m MD': the depth at which new formation is first reported is not separable inside the interval, so the first tier gives no point value; the second tier gives where the kick-off drilling started, 2,531 m. The sidetrack's first report starts at 2,627 m, so 2,589 m is not supported either. NOD 2,586 m and 2,589 m both lie inside the interval, so the uncertainty is about 58 m.</t>
-        </is>
-      </c>
-      <c r="R12" s="4" t="n"/>
-      <c r="S12" s="4" t="n"/>
-      <c r="T12" s="4" t="n"/>
+          <t>LOW confidence. 'Drilled cement and new formation from 2531 m MD to 2589 m MD' reports new formation by the end of the interval, so departure is confirmed at 2,589 m, consistent with F-1 C (formation first reported); the interval start, 2,531 m, is not used (TJ ruling, decision 40). NOD gives 2,586 m, inside the interval.</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="n">
+        <v>2589</v>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>LOW confidence. 'Drilled cement and new formation from 2531 m MD to 2589 m MD' reports new formation by the end of the interval, so departure is confirmed at 2,589 m, consistent with F-1 C (formation first reported); the interval start, 2,531 m, is not used (TJ ruling, decision 40). NOD gives 2,586 m, inside the interval.</t>
+        </is>
+      </c>
+      <c r="V12" s="4" t="n"/>
+      <c r="W12" s="4" t="n"/>
+      <c r="X12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1483,9 +1705,27 @@
           <t>'Drilled cement/new formation from 1368 m to 1381 m MD. Initiated kick off of F-15.' puts the start of the kick-off at the end of the interval, 1,381 m, where the sidetrack's first report also starts. NOD agrees at 1,381 m.</t>
         </is>
       </c>
-      <c r="R13" s="4" t="n"/>
-      <c r="S13" s="4" t="n"/>
-      <c r="T13" s="4" t="n"/>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="n">
+        <v>1381</v>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>'Drilled cement/new formation from 1368 m to 1381 m MD. Initiated kick off of F-15.' puts the start of the kick-off at the end of the interval, 1,381 m, where the sidetrack's first report also starts. NOD agrees at 1,381 m.</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="n"/>
+      <c r="W13" s="4" t="n"/>
+      <c r="X13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1559,9 +1799,27 @@
           <t>Tier 1: 'kicked off at 3185m' states the departure depth; the '50/50 cement/formation' remark relates to 3,210 m, drilled afterwards. NOD agrees at 3,185 m.</t>
         </is>
       </c>
-      <c r="R14" s="4" t="n"/>
-      <c r="S14" s="4" t="n"/>
-      <c r="T14" s="4" t="n"/>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="n">
+        <v>3185</v>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>Tier 1: 'kicked off at 3185m' states the departure depth; the '50/50 cement/formation' remark relates to 3,210 m, drilled afterwards. NOD agrees at 3,185 m.</t>
+        </is>
+      </c>
+      <c r="V14" s="4" t="n"/>
+      <c r="W14" s="4" t="n"/>
+      <c r="X14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1639,9 +1897,27 @@
           <t>Tier 2: cement was drilled from 2,490 to 2,566 m, then 'Initiated kick off', and no formation or departure depth is stated; 2,575 m (the NOD value) is only where the section had reached by the end of the day.</t>
         </is>
       </c>
-      <c r="R15" s="4" t="n"/>
-      <c r="S15" s="4" t="n"/>
-      <c r="T15" s="4" t="n"/>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="n">
+        <v>2566</v>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>Tier 2: cement was drilled from 2,490 to 2,566 m, then 'Initiated kick off', and no formation or departure depth is stated; 2,575 m (the NOD value) is only where the section had reached by the end of the day.</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="n"/>
+      <c r="W15" s="4" t="n"/>
+      <c r="X15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1715,13 +1991,31 @@
           <t>The sidetrack's first report says 'Drilled cement and kicked off' without a depth, so tier 2 with depth from md: the parent's last report (kick-off plug set the day before) has md 1,380 m. NOD agrees at 1,380 m.</t>
         </is>
       </c>
-      <c r="R16" s="4" t="n"/>
-      <c r="S16" s="4" t="n"/>
-      <c r="T16" s="4" t="n"/>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="n">
+        <v>1380</v>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>The sidetrack's first report says 'Drilled cement and kicked off' without a depth, so tier 2 with depth from md: the parent's last report (kick-off plug set the day before) has md 1,380 m. NOD agrees at 1,380 m.</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="n"/>
+      <c r="W16" s="4" t="n"/>
+      <c r="X16" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="O2:O16 R2:R16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="S2:S16 V2:V16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>